<commit_message>
fix: add aboslute protein volume analysis
</commit_message>
<xml_diff>
--- a/data/proteomics/organell_protein_volume_tao2.xlsx
+++ b/data/proteomics/organell_protein_volume_tao2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EK9"/>
+  <dimension ref="A1:EM9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1129,6 +1129,16 @@
           <t>sample_ID</t>
         </is>
       </c>
+      <c r="EL1" s="1" t="inlineStr">
+        <is>
+          <t>total_pro_volume</t>
+        </is>
+      </c>
+      <c r="EM1" s="1" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -1556,6 +1566,14 @@
       <c r="EK2" t="n">
         <v>5</v>
       </c>
+      <c r="EL2" t="n">
+        <v>1.912475495650298</v>
+      </c>
+      <c r="EM2" t="inlineStr">
+        <is>
+          <t>C-lim rep1 prot (fmol mgDW-1)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -1983,6 +2001,14 @@
       <c r="EK3" t="n">
         <v>5</v>
       </c>
+      <c r="EL3" t="n">
+        <v>1.967840779985522</v>
+      </c>
+      <c r="EM3" t="inlineStr">
+        <is>
+          <t>C-lim rep2 prot (fmol mgDW-1)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -2410,6 +2436,14 @@
       <c r="EK4" t="n">
         <v>115</v>
       </c>
+      <c r="EL4" t="n">
+        <v>0.9861729177512535</v>
+      </c>
+      <c r="EM4" t="inlineStr">
+        <is>
+          <t>C/N=115 rep1 prot (fmol mgDW-1)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -2837,6 +2871,14 @@
       <c r="EK5" t="n">
         <v>115</v>
       </c>
+      <c r="EL5" t="n">
+        <v>1.127757767916389</v>
+      </c>
+      <c r="EM5" t="inlineStr">
+        <is>
+          <t>C/N=115 rep2 prot (fmol mgDW-1)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -3264,6 +3306,14 @@
       <c r="EK6" t="n">
         <v>30</v>
       </c>
+      <c r="EL6" t="n">
+        <v>1.488678410143015</v>
+      </c>
+      <c r="EM6" t="inlineStr">
+        <is>
+          <t>C/N=30 rep1 prot (fmol mgDW-1)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -3691,6 +3741,14 @@
       <c r="EK7" t="n">
         <v>30</v>
       </c>
+      <c r="EL7" t="n">
+        <v>1.520156369982094</v>
+      </c>
+      <c r="EM7" t="inlineStr">
+        <is>
+          <t>C/N=30 rep2 prot (fmol mgDW-1)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -4118,6 +4176,14 @@
       <c r="EK8" t="n">
         <v>50</v>
       </c>
+      <c r="EL8" t="n">
+        <v>0.8921217673791332</v>
+      </c>
+      <c r="EM8" t="inlineStr">
+        <is>
+          <t>C/N=50 rep1 prot (fmol mgDW-1)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -4544,6 +4610,14 @@
       </c>
       <c r="EK9" t="n">
         <v>50</v>
+      </c>
+      <c r="EL9" t="n">
+        <v>0.9292315671910052</v>
+      </c>
+      <c r="EM9" t="inlineStr">
+        <is>
+          <t>C/N=50 rep2 prot (fmol mgDW-1)</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>